<commit_message>
Costa Atlantica y seccion del informe INECO
- Electricidad de las cooperativas de Villa Gesell y San Bernardo (CAMMESA): temporada (ene-feb) vs
  invierno (jun-ago) comparadas con el total del pais; grafico 11 y seccion nueva en el notebook 02
- docs/informe_indicadores/seccion_energia.tex: seccion para la Propuesta de Indicadores Economicos
  (indice nacional, provincias y propuesta de foco en Pinamar y General Madariaga)
- ESTADO: Colab verificado con 0b9f55a, cifras de la Costa Atlantica
</commit_message>
<xml_diff>
--- a/output/indice_consumo_energetico.xlsx
+++ b/output/indice_consumo_energetico.xlsx
@@ -20,7 +20,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ramas_gas_TJ_anual" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ramas_gas_indice_12m" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gas_m3_por_usuario" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarifas_CAMMESA" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Costa_resumen" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Costa_GWh_mensual" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Costa_temporadas_indice" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarifas_CAMMESA" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -53,7 +56,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -66,6 +69,34 @@
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -462,7 +493,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Version del codigo (commit): f7926c2 (2026-10-07)</t>
+          <t>Version del codigo (commit): 0b9f55a (2026-10-07)</t>
         </is>
       </c>
     </row>
@@ -26306,6 +26337,3450 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>localidad</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>gwh_2025</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>part_hogares_2025_%</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>enero_vs_promedio</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>verano_2026_vs_2025_%</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>verano_2026_vs_2016_%</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>invierno_2026_vs_2025_%</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>invierno_2026_vs_2016_%</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>verano_sobre_invierno_2016</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>verano_sobre_invierno_2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>San Bernardo (La Costa)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>47.889863</v>
+      </c>
+      <c r="C2" t="n">
+        <v>53.62741171341417</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2.069635571466236</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-2.078014787536631</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-31.89509554869987</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.3458593169062718</v>
+      </c>
+      <c r="H2" t="n">
+        <v>24.29884608940272</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3.077882186036668</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1.686410443759199</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Total país</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>141250.903437</v>
+      </c>
+      <c r="C3" t="n">
+        <v>47.00289369802992</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.111043310497497</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-5.987803800623571</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3.52719423480603</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2.22727060911061</v>
+      </c>
+      <c r="H3" t="n">
+        <v>10.22711020355604</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1.043849338403702</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.9804012189853046</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Villa Gesell</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>150.578415</v>
+      </c>
+      <c r="C4" t="n">
+        <v>64.81372977660841</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.432523121140906</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-2.530974234121974</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-2.160143109338097</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.4478928509036528</v>
+      </c>
+      <c r="H4" t="n">
+        <v>17.95234463403119</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1.341496183363939</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1.1127527393112</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D177"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>San Bernardo (La Costa)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Total país</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Villa Gesell</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>2012-01</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>7.148264</v>
+      </c>
+      <c r="C2" t="n">
+        <v>10804.699842</v>
+      </c>
+      <c r="D2" t="n">
+        <v>15.718099</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>2012-02</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>6.125955</v>
+      </c>
+      <c r="C3" t="n">
+        <v>10085.552231</v>
+      </c>
+      <c r="D3" t="n">
+        <v>13.81417</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>2012-03</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3.327711</v>
+      </c>
+      <c r="C4" t="n">
+        <v>10175.365005</v>
+      </c>
+      <c r="D4" t="n">
+        <v>9.574142999999999</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>2012-04</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2.841553</v>
+      </c>
+      <c r="C5" t="n">
+        <v>8969.068409</v>
+      </c>
+      <c r="D5" t="n">
+        <v>9.285671000000001</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>2012-05</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2.483421</v>
+      </c>
+      <c r="C6" t="n">
+        <v>9597.272015999999</v>
+      </c>
+      <c r="D6" t="n">
+        <v>9.236225000000001</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>2012-06</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2.504562</v>
+      </c>
+      <c r="C7" t="n">
+        <v>10292.182399</v>
+      </c>
+      <c r="D7" t="n">
+        <v>9.934833000000001</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>2012-07</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3.154724</v>
+      </c>
+      <c r="C8" t="n">
+        <v>11066.530786</v>
+      </c>
+      <c r="D8" t="n">
+        <v>12.160697</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>2012-08</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2.632021</v>
+      </c>
+      <c r="C9" t="n">
+        <v>10404.120825</v>
+      </c>
+      <c r="D9" t="n">
+        <v>10.464223</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>2012-09</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2.519386</v>
+      </c>
+      <c r="C10" t="n">
+        <v>9336.891496</v>
+      </c>
+      <c r="D10" t="n">
+        <v>9.374686000000001</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>2012-10</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2.489281000000001</v>
+      </c>
+      <c r="C11" t="n">
+        <v>9608.256140000001</v>
+      </c>
+      <c r="D11" t="n">
+        <v>8.960726999999999</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>2012-11</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2.497439</v>
+      </c>
+      <c r="C12" t="n">
+        <v>10027.740717</v>
+      </c>
+      <c r="D12" t="n">
+        <v>7.974638000000001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>2012-12</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>3.511304</v>
+      </c>
+      <c r="C13" t="n">
+        <v>10820.739305</v>
+      </c>
+      <c r="D13" t="n">
+        <v>9.970445</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>2013-01</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>7.083452</v>
+      </c>
+      <c r="C14" t="n">
+        <v>11134.119345</v>
+      </c>
+      <c r="D14" t="n">
+        <v>15.896856</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>2013-02</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>5.824619999999999</v>
+      </c>
+      <c r="C15" t="n">
+        <v>9834.160006999999</v>
+      </c>
+      <c r="D15" t="n">
+        <v>13.41278</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>2013-03</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3.601310999999999</v>
+      </c>
+      <c r="C16" t="n">
+        <v>9756.129308</v>
+      </c>
+      <c r="D16" t="n">
+        <v>10.399227</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>2013-04</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2.527857</v>
+      </c>
+      <c r="C17" t="n">
+        <v>9307.334163000001</v>
+      </c>
+      <c r="D17" t="n">
+        <v>8.438461999999999</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>2013-05</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2.534502</v>
+      </c>
+      <c r="C18" t="n">
+        <v>10232.825394</v>
+      </c>
+      <c r="D18" t="n">
+        <v>9.678921000000001</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>2013-06</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2.806329</v>
+      </c>
+      <c r="C19" t="n">
+        <v>10360.537194</v>
+      </c>
+      <c r="D19" t="n">
+        <v>10.941133</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>2013-07</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3.130516</v>
+      </c>
+      <c r="C20" t="n">
+        <v>11156.173393</v>
+      </c>
+      <c r="D20" t="n">
+        <v>12.027874</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>2013-08</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2.825832</v>
+      </c>
+      <c r="C21" t="n">
+        <v>10904.479243</v>
+      </c>
+      <c r="D21" t="n">
+        <v>10.989579</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>2013-09</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2.555652</v>
+      </c>
+      <c r="C22" t="n">
+        <v>10195.872995</v>
+      </c>
+      <c r="D22" t="n">
+        <v>9.866292</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>2013-10</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2.552566</v>
+      </c>
+      <c r="C23" t="n">
+        <v>10045.715632</v>
+      </c>
+      <c r="D23" t="n">
+        <v>9.164901</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>2013-11</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2.53848</v>
+      </c>
+      <c r="C24" t="n">
+        <v>10015.701652</v>
+      </c>
+      <c r="D24" t="n">
+        <v>8.546147999999999</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>2013-12</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>3.709319</v>
+      </c>
+      <c r="C25" t="n">
+        <v>12291.286493</v>
+      </c>
+      <c r="D25" t="n">
+        <v>11.026209</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>2014-01</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>7.865305999999999</v>
+      </c>
+      <c r="C26" t="n">
+        <v>12004.342368</v>
+      </c>
+      <c r="D26" t="n">
+        <v>16.578157</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>2014-02</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>7.566059999999999</v>
+      </c>
+      <c r="C27" t="n">
+        <v>9823.968201</v>
+      </c>
+      <c r="D27" t="n">
+        <v>13.410231</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>2014-03</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>3.920143</v>
+      </c>
+      <c r="C28" t="n">
+        <v>9789.798789</v>
+      </c>
+      <c r="D28" t="n">
+        <v>10.297739</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>2014-04</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>2.723989</v>
+      </c>
+      <c r="C29" t="n">
+        <v>9595.37435</v>
+      </c>
+      <c r="D29" t="n">
+        <v>9.255732999999999</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>2014-05</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>2.653838</v>
+      </c>
+      <c r="C30" t="n">
+        <v>10409.105006</v>
+      </c>
+      <c r="D30" t="n">
+        <v>9.795986000000001</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>2014-06</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>2.660122</v>
+      </c>
+      <c r="C31" t="n">
+        <v>10901.714976</v>
+      </c>
+      <c r="D31" t="n">
+        <v>10.259386</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>2014-07</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>2.916715</v>
+      </c>
+      <c r="C32" t="n">
+        <v>11363.942102</v>
+      </c>
+      <c r="D32" t="n">
+        <v>11.513832</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>2014-08</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2.719495</v>
+      </c>
+      <c r="C33" t="n">
+        <v>10490.682389</v>
+      </c>
+      <c r="D33" t="n">
+        <v>10.543369</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>2014-09</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>2.3333</v>
+      </c>
+      <c r="C34" t="n">
+        <v>9807.544190999999</v>
+      </c>
+      <c r="D34" t="n">
+        <v>9.133232</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>2014-10</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>2.541587</v>
+      </c>
+      <c r="C35" t="n">
+        <v>10706.493141</v>
+      </c>
+      <c r="D35" t="n">
+        <v>9.087382999999999</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>2014-11</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>2.575247</v>
+      </c>
+      <c r="C36" t="n">
+        <v>10344.736672</v>
+      </c>
+      <c r="D36" t="n">
+        <v>8.548303000000001</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>2014-12</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>3.758906</v>
+      </c>
+      <c r="C37" t="n">
+        <v>11229.37782</v>
+      </c>
+      <c r="D37" t="n">
+        <v>11.173843</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>2015-01</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>9.602209999999999</v>
+      </c>
+      <c r="C38" t="n">
+        <v>11706.190093</v>
+      </c>
+      <c r="D38" t="n">
+        <v>16.715774</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>2015-02</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>8.170799000000001</v>
+      </c>
+      <c r="C39" t="n">
+        <v>10665.086621</v>
+      </c>
+      <c r="D39" t="n">
+        <v>14.452197</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>2015-03</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>3.945573</v>
+      </c>
+      <c r="C40" t="n">
+        <v>11548.527072</v>
+      </c>
+      <c r="D40" t="n">
+        <v>11.276745</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>2015-04</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2.73291</v>
+      </c>
+      <c r="C41" t="n">
+        <v>10026.43476</v>
+      </c>
+      <c r="D41" t="n">
+        <v>8.978633</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>2015-05</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>2.63164</v>
+      </c>
+      <c r="C42" t="n">
+        <v>10467.633693</v>
+      </c>
+      <c r="D42" t="n">
+        <v>9.948514000000001</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>2015-06</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2.629802</v>
+      </c>
+      <c r="C43" t="n">
+        <v>11254.419667</v>
+      </c>
+      <c r="D43" t="n">
+        <v>10.634843</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>2015-07</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>3.123951</v>
+      </c>
+      <c r="C44" t="n">
+        <v>11907.361919</v>
+      </c>
+      <c r="D44" t="n">
+        <v>12.305295</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>2015-08</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2.736359</v>
+      </c>
+      <c r="C45" t="n">
+        <v>11130.262808</v>
+      </c>
+      <c r="D45" t="n">
+        <v>11.192609</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>2015-09</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2.544394</v>
+      </c>
+      <c r="C46" t="n">
+        <v>10552.903241</v>
+      </c>
+      <c r="D46" t="n">
+        <v>10.25443</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>2015-10</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2.815926</v>
+      </c>
+      <c r="C47" t="n">
+        <v>10722.174389</v>
+      </c>
+      <c r="D47" t="n">
+        <v>10.866434</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>2015-11</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2.564091</v>
+      </c>
+      <c r="C48" t="n">
+        <v>10219.189482</v>
+      </c>
+      <c r="D48" t="n">
+        <v>8.872457000000001</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>2015-12</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>4.756936</v>
+      </c>
+      <c r="C49" t="n">
+        <v>11909.435561</v>
+      </c>
+      <c r="D49" t="n">
+        <v>11.794942</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>2016-01</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>9.973002999999999</v>
+      </c>
+      <c r="C50" t="n">
+        <v>12344.911762</v>
+      </c>
+      <c r="D50" t="n">
+        <v>16.664968</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>2016-02</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>8.641536</v>
+      </c>
+      <c r="C51" t="n">
+        <v>11731.845101</v>
+      </c>
+      <c r="D51" t="n">
+        <v>14.824242</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>2016-03</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>3.745157</v>
+      </c>
+      <c r="C52" t="n">
+        <v>10461.47592</v>
+      </c>
+      <c r="D52" t="n">
+        <v>10.729283</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>2016-04</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2.61245</v>
+      </c>
+      <c r="C53" t="n">
+        <v>10292.000856</v>
+      </c>
+      <c r="D53" t="n">
+        <v>9.21547</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>2016-05</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>2.840681</v>
+      </c>
+      <c r="C54" t="n">
+        <v>11358.011628</v>
+      </c>
+      <c r="D54" t="n">
+        <v>10.917297</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>2016-06</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>2.905066</v>
+      </c>
+      <c r="C55" t="n">
+        <v>11812.94705</v>
+      </c>
+      <c r="D55" t="n">
+        <v>11.462226</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>2016-07</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>3.270836</v>
+      </c>
+      <c r="C56" t="n">
+        <v>11929.645375</v>
+      </c>
+      <c r="D56" t="n">
+        <v>12.580206</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>2016-08</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2.895858</v>
+      </c>
+      <c r="C57" t="n">
+        <v>10855.441952</v>
+      </c>
+      <c r="D57" t="n">
+        <v>11.16737</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t>2016-09</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>2.631402</v>
+      </c>
+      <c r="C58" t="n">
+        <v>10382.081134</v>
+      </c>
+      <c r="D58" t="n">
+        <v>10.058709</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="inlineStr">
+        <is>
+          <t>2016-10</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>2.746337</v>
+      </c>
+      <c r="C59" t="n">
+        <v>9956.038875</v>
+      </c>
+      <c r="D59" t="n">
+        <v>9.910718000000001</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="inlineStr">
+        <is>
+          <t>2016-11</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>2.751039</v>
+      </c>
+      <c r="C60" t="n">
+        <v>10132.540584</v>
+      </c>
+      <c r="D60" t="n">
+        <v>8.659889999999999</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="inlineStr">
+        <is>
+          <t>2016-12</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>4.295599</v>
+      </c>
+      <c r="C61" t="n">
+        <v>11853.854388</v>
+      </c>
+      <c r="D61" t="n">
+        <v>11.249453</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="inlineStr">
+        <is>
+          <t>2017-01</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>9.301054000000001</v>
+      </c>
+      <c r="C62" t="n">
+        <v>12524.865646</v>
+      </c>
+      <c r="D62" t="n">
+        <v>16.208871</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t>2017-02</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>8.227596</v>
+      </c>
+      <c r="C63" t="n">
+        <v>11074.906499</v>
+      </c>
+      <c r="D63" t="n">
+        <v>13.597201</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="inlineStr">
+        <is>
+          <t>2017-03</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>4.276801000000001</v>
+      </c>
+      <c r="C64" t="n">
+        <v>11122.231555</v>
+      </c>
+      <c r="D64" t="n">
+        <v>10.251095</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="inlineStr">
+        <is>
+          <t>2017-04</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>2.844479</v>
+      </c>
+      <c r="C65" t="n">
+        <v>9793.758585000001</v>
+      </c>
+      <c r="D65" t="n">
+        <v>9.416189000000001</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="inlineStr">
+        <is>
+          <t>2017-05</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>2.640809</v>
+      </c>
+      <c r="C66" t="n">
+        <v>10795.213415</v>
+      </c>
+      <c r="D66" t="n">
+        <v>9.744139000000001</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="inlineStr">
+        <is>
+          <t>2017-06</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>2.767734</v>
+      </c>
+      <c r="C67" t="n">
+        <v>11359.330662</v>
+      </c>
+      <c r="D67" t="n">
+        <v>10.91949</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="inlineStr">
+        <is>
+          <t>2017-07</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>3.277193</v>
+      </c>
+      <c r="C68" t="n">
+        <v>11796.425757</v>
+      </c>
+      <c r="D68" t="n">
+        <v>12.441057</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="inlineStr">
+        <is>
+          <t>2017-08</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>2.974484</v>
+      </c>
+      <c r="C69" t="n">
+        <v>11107.250705</v>
+      </c>
+      <c r="D69" t="n">
+        <v>11.087275</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="inlineStr">
+        <is>
+          <t>2017-09</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>2.662154</v>
+      </c>
+      <c r="C70" t="n">
+        <v>10348.584548</v>
+      </c>
+      <c r="D70" t="n">
+        <v>9.789389</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="inlineStr">
+        <is>
+          <t>2017-10</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>2.666313</v>
+      </c>
+      <c r="C71" t="n">
+        <v>10227.329313</v>
+      </c>
+      <c r="D71" t="n">
+        <v>9.307733999999998</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="inlineStr">
+        <is>
+          <t>2017-11</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>2.733213</v>
+      </c>
+      <c r="C72" t="n">
+        <v>10355.727486</v>
+      </c>
+      <c r="D72" t="n">
+        <v>8.803125</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="inlineStr">
+        <is>
+          <t>2017-12</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>3.918469</v>
+      </c>
+      <c r="C73" t="n">
+        <v>12024.595461</v>
+      </c>
+      <c r="D73" t="n">
+        <v>10.941149</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="inlineStr">
+        <is>
+          <t>2018-01</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>9.366965</v>
+      </c>
+      <c r="C74" t="n">
+        <v>12350.18332</v>
+      </c>
+      <c r="D74" t="n">
+        <v>16.442052</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="inlineStr">
+        <is>
+          <t>2018-02</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>7.46835</v>
+      </c>
+      <c r="C75" t="n">
+        <v>11404.202882</v>
+      </c>
+      <c r="D75" t="n">
+        <v>14.541698</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="inlineStr">
+        <is>
+          <t>2018-03</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>3.891489</v>
+      </c>
+      <c r="C76" t="n">
+        <v>11247.242133</v>
+      </c>
+      <c r="D76" t="n">
+        <v>10.898343</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="inlineStr">
+        <is>
+          <t>2018-04</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>2.853946</v>
+      </c>
+      <c r="C77" t="n">
+        <v>10493.314585</v>
+      </c>
+      <c r="D77" t="n">
+        <v>9.148019999999999</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="inlineStr">
+        <is>
+          <t>2018-05</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>2.819546</v>
+      </c>
+      <c r="C78" t="n">
+        <v>10665.461507</v>
+      </c>
+      <c r="D78" t="n">
+        <v>10.013771</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="inlineStr">
+        <is>
+          <t>2018-06</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>2.858826</v>
+      </c>
+      <c r="C79" t="n">
+        <v>11925.613707</v>
+      </c>
+      <c r="D79" t="n">
+        <v>11.294693</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="inlineStr">
+        <is>
+          <t>2018-07</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>3.371124</v>
+      </c>
+      <c r="C80" t="n">
+        <v>12607.552722</v>
+      </c>
+      <c r="D80" t="n">
+        <v>13.127669</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="inlineStr">
+        <is>
+          <t>2018-08</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>2.948678</v>
+      </c>
+      <c r="C81" t="n">
+        <v>11720.547081</v>
+      </c>
+      <c r="D81" t="n">
+        <v>11.599327</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="inlineStr">
+        <is>
+          <t>2018-09</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>2.476127</v>
+      </c>
+      <c r="C82" t="n">
+        <v>9777.819303999999</v>
+      </c>
+      <c r="D82" t="n">
+        <v>9.608308999999998</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="inlineStr">
+        <is>
+          <t>2018-10</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>2.592919</v>
+      </c>
+      <c r="C83" t="n">
+        <v>9895.852265000001</v>
+      </c>
+      <c r="D83" t="n">
+        <v>9.4956</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="inlineStr">
+        <is>
+          <t>2018-11</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>2.662212</v>
+      </c>
+      <c r="C84" t="n">
+        <v>10029.029749</v>
+      </c>
+      <c r="D84" t="n">
+        <v>8.653221</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="inlineStr">
+        <is>
+          <t>2018-12</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>3.615762</v>
+      </c>
+      <c r="C85" t="n">
+        <v>10808.319667</v>
+      </c>
+      <c r="D85" t="n">
+        <v>10.473017</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="inlineStr">
+        <is>
+          <t>2019-01</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>8.307026</v>
+      </c>
+      <c r="C86" t="n">
+        <v>11698.820402</v>
+      </c>
+      <c r="D86" t="n">
+        <v>15.879793</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="inlineStr">
+        <is>
+          <t>2019-02</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>5.763836</v>
+      </c>
+      <c r="C87" t="n">
+        <v>10706.955317</v>
+      </c>
+      <c r="D87" t="n">
+        <v>13.723382</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="inlineStr">
+        <is>
+          <t>2019-03</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>3.606097</v>
+      </c>
+      <c r="C88" t="n">
+        <v>10120.057936</v>
+      </c>
+      <c r="D88" t="n">
+        <v>10.205401</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="inlineStr">
+        <is>
+          <t>2019-04</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>2.675233</v>
+      </c>
+      <c r="C89" t="n">
+        <v>9572.130644999999</v>
+      </c>
+      <c r="D89" t="n">
+        <v>8.395095999999999</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="1" t="inlineStr">
+        <is>
+          <t>2019-05</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>2.57385</v>
+      </c>
+      <c r="C90" t="n">
+        <v>10382.062156</v>
+      </c>
+      <c r="D90" t="n">
+        <v>9.222119000000001</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="inlineStr">
+        <is>
+          <t>2019-06</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>2.627332</v>
+      </c>
+      <c r="C91" t="n">
+        <v>10649.85454</v>
+      </c>
+      <c r="D91" t="n">
+        <v>9.869221</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="inlineStr">
+        <is>
+          <t>2019-07</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>3.327234999999999</v>
+      </c>
+      <c r="C92" t="n">
+        <v>12004.210188</v>
+      </c>
+      <c r="D92" t="n">
+        <v>8.149940000000001</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="inlineStr">
+        <is>
+          <t>2019-08</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>2.798094</v>
+      </c>
+      <c r="C93" t="n">
+        <v>11465.483299</v>
+      </c>
+      <c r="D93" t="n">
+        <v>11.296616</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="inlineStr">
+        <is>
+          <t>2019-09</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>2.094555</v>
+      </c>
+      <c r="C94" t="n">
+        <v>10218.087823</v>
+      </c>
+      <c r="D94" t="n">
+        <v>9.920855000000001</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="1" t="inlineStr">
+        <is>
+          <t>2019-10</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>1.77933</v>
+      </c>
+      <c r="C95" t="n">
+        <v>10380.686879</v>
+      </c>
+      <c r="D95" t="n">
+        <v>9.429234000000001</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="1" t="inlineStr">
+        <is>
+          <t>2019-11</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>2.203678</v>
+      </c>
+      <c r="C96" t="n">
+        <v>10559.966155</v>
+      </c>
+      <c r="D96" t="n">
+        <v>8.257785999999999</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="1" t="inlineStr">
+        <is>
+          <t>2019-12</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>2.728924</v>
+      </c>
+      <c r="C97" t="n">
+        <v>11187.742677</v>
+      </c>
+      <c r="D97" t="n">
+        <v>10.365577</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="1" t="inlineStr">
+        <is>
+          <t>2020-01</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>6.843051</v>
+      </c>
+      <c r="C98" t="n">
+        <v>11993.867057</v>
+      </c>
+      <c r="D98" t="n">
+        <v>16.079791</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="1" t="inlineStr">
+        <is>
+          <t>2020-02</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>6.155024999999999</v>
+      </c>
+      <c r="C99" t="n">
+        <v>10843.47443</v>
+      </c>
+      <c r="D99" t="n">
+        <v>14.495323</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="1" t="inlineStr">
+        <is>
+          <t>2020-03</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>3.274614</v>
+      </c>
+      <c r="C100" t="n">
+        <v>11144.232192</v>
+      </c>
+      <c r="D100" t="n">
+        <v>9.678205999999999</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="1" t="inlineStr">
+        <is>
+          <t>2020-04</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>2.176572</v>
+      </c>
+      <c r="C101" t="n">
+        <v>8537.200407</v>
+      </c>
+      <c r="D101" t="n">
+        <v>7.895417</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="1" t="inlineStr">
+        <is>
+          <t>2020-05</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>2.432602</v>
+      </c>
+      <c r="C102" t="n">
+        <v>9617.328172</v>
+      </c>
+      <c r="D102" t="n">
+        <v>9.365843999999999</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="1" t="inlineStr">
+        <is>
+          <t>2020-06</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>2.666178</v>
+      </c>
+      <c r="C103" t="n">
+        <v>10781.714873</v>
+      </c>
+      <c r="D103" t="n">
+        <v>10.238635</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="1" t="inlineStr">
+        <is>
+          <t>2020-07</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>2.999914</v>
+      </c>
+      <c r="C104" t="n">
+        <v>12183.852641</v>
+      </c>
+      <c r="D104" t="n">
+        <v>11.542367</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="1" t="inlineStr">
+        <is>
+          <t>2020-08</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>2.813273</v>
+      </c>
+      <c r="C105" t="n">
+        <v>10728.379158</v>
+      </c>
+      <c r="D105" t="n">
+        <v>10.563111</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="1" t="inlineStr">
+        <is>
+          <t>2020-09</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>2.501684</v>
+      </c>
+      <c r="C106" t="n">
+        <v>10045.02285</v>
+      </c>
+      <c r="D106" t="n">
+        <v>9.585519</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="1" t="inlineStr">
+        <is>
+          <t>2020-10</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>2.339918</v>
+      </c>
+      <c r="C107" t="n">
+        <v>10013.844018</v>
+      </c>
+      <c r="D107" t="n">
+        <v>8.727012</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="1" t="inlineStr">
+        <is>
+          <t>2020-11</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>2.282615</v>
+      </c>
+      <c r="C108" t="n">
+        <v>10087.844439</v>
+      </c>
+      <c r="D108" t="n">
+        <v>7.610640999999999</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="1" t="inlineStr">
+        <is>
+          <t>2020-12</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>3.296352</v>
+      </c>
+      <c r="C109" t="n">
+        <v>11330.177614</v>
+      </c>
+      <c r="D109" t="n">
+        <v>10.52948</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="1" t="inlineStr">
+        <is>
+          <t>2021-01</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>5.061955000000001</v>
+      </c>
+      <c r="C110" t="n">
+        <v>11941.580986</v>
+      </c>
+      <c r="D110" t="n">
+        <v>13.780138</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="1" t="inlineStr">
+        <is>
+          <t>2021-02</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>4.451404999999999</v>
+      </c>
+      <c r="C111" t="n">
+        <v>10090.389298</v>
+      </c>
+      <c r="D111" t="n">
+        <v>11.734417</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="1" t="inlineStr">
+        <is>
+          <t>2021-03</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>3.395292</v>
+      </c>
+      <c r="C112" t="n">
+        <v>11055.214503</v>
+      </c>
+      <c r="D112" t="n">
+        <v>10.27912</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="1" t="inlineStr">
+        <is>
+          <t>2021-04</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>2.578226</v>
+      </c>
+      <c r="C113" t="n">
+        <v>9817.737877</v>
+      </c>
+      <c r="D113" t="n">
+        <v>8.554876</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="1" t="inlineStr">
+        <is>
+          <t>2021-05</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>2.773494</v>
+      </c>
+      <c r="C114" t="n">
+        <v>10986.114068</v>
+      </c>
+      <c r="D114" t="n">
+        <v>10.599732</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="1" t="inlineStr">
+        <is>
+          <t>2021-06</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>2.985875</v>
+      </c>
+      <c r="C115" t="n">
+        <v>12053.804232</v>
+      </c>
+      <c r="D115" t="n">
+        <v>11.547947</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="1" t="inlineStr">
+        <is>
+          <t>2021-07</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>3.587746</v>
+      </c>
+      <c r="C116" t="n">
+        <v>12418.960365</v>
+      </c>
+      <c r="D116" t="n">
+        <v>13.714007</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="1" t="inlineStr">
+        <is>
+          <t>2021-08</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>3.314819</v>
+      </c>
+      <c r="C117" t="n">
+        <v>11660.287778</v>
+      </c>
+      <c r="D117" t="n">
+        <v>12.580778</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="1" t="inlineStr">
+        <is>
+          <t>2021-09</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>2.897514</v>
+      </c>
+      <c r="C118" t="n">
+        <v>10374.79406</v>
+      </c>
+      <c r="D118" t="n">
+        <v>10.59468</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="1" t="inlineStr">
+        <is>
+          <t>2021-10</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>3.046022</v>
+      </c>
+      <c r="C119" t="n">
+        <v>10451.324175</v>
+      </c>
+      <c r="D119" t="n">
+        <v>10.670088</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="1" t="inlineStr">
+        <is>
+          <t>2021-11</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>2.891751</v>
+      </c>
+      <c r="C120" t="n">
+        <v>10569.433719</v>
+      </c>
+      <c r="D120" t="n">
+        <v>9.391813000000001</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="1" t="inlineStr">
+        <is>
+          <t>2021-12</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>3.830255</v>
+      </c>
+      <c r="C121" t="n">
+        <v>12457.126697</v>
+      </c>
+      <c r="D121" t="n">
+        <v>11.617377</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="1" t="inlineStr">
+        <is>
+          <t>2022-01</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>6.994505</v>
+      </c>
+      <c r="C122" t="n">
+        <v>13065.875758</v>
+      </c>
+      <c r="D122" t="n">
+        <v>17.239671</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="1" t="inlineStr">
+        <is>
+          <t>2022-02</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>5.58512</v>
+      </c>
+      <c r="C123" t="n">
+        <v>10566.724241</v>
+      </c>
+      <c r="D123" t="n">
+        <v>13.849346</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="1" t="inlineStr">
+        <is>
+          <t>2022-03</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>3.741032</v>
+      </c>
+      <c r="C124" t="n">
+        <v>10880.355192</v>
+      </c>
+      <c r="D124" t="n">
+        <v>11.158794</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="1" t="inlineStr">
+        <is>
+          <t>2022-04</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>3.043315</v>
+      </c>
+      <c r="C125" t="n">
+        <v>10146.368066</v>
+      </c>
+      <c r="D125" t="n">
+        <v>10.442161</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="1" t="inlineStr">
+        <is>
+          <t>2022-05</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>3.136419000000001</v>
+      </c>
+      <c r="C126" t="n">
+        <v>11726.718022</v>
+      </c>
+      <c r="D126" t="n">
+        <v>11.945089</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="1" t="inlineStr">
+        <is>
+          <t>2022-06</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>3.640101</v>
+      </c>
+      <c r="C127" t="n">
+        <v>13073.296211</v>
+      </c>
+      <c r="D127" t="n">
+        <v>14.101677</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="1" t="inlineStr">
+        <is>
+          <t>2022-07</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>3.885443</v>
+      </c>
+      <c r="C128" t="n">
+        <v>12638.511304</v>
+      </c>
+      <c r="D128" t="n">
+        <v>14.967132</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="1" t="inlineStr">
+        <is>
+          <t>2022-08</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>3.38149</v>
+      </c>
+      <c r="C129" t="n">
+        <v>11781.464254</v>
+      </c>
+      <c r="D129" t="n">
+        <v>13.194182</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="1" t="inlineStr">
+        <is>
+          <t>2022-09</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>2.937171</v>
+      </c>
+      <c r="C130" t="n">
+        <v>10311.68584</v>
+      </c>
+      <c r="D130" t="n">
+        <v>11.129838</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="1" t="inlineStr">
+        <is>
+          <t>2022-10</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>3.199738</v>
+      </c>
+      <c r="C131" t="n">
+        <v>10217.226992</v>
+      </c>
+      <c r="D131" t="n">
+        <v>11.395923</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="1" t="inlineStr">
+        <is>
+          <t>2022-11</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>2.997689</v>
+      </c>
+      <c r="C132" t="n">
+        <v>11322.091207</v>
+      </c>
+      <c r="D132" t="n">
+        <v>9.683152</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="1" t="inlineStr">
+        <is>
+          <t>2022-12</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>3.985913</v>
+      </c>
+      <c r="C133" t="n">
+        <v>13024.74442</v>
+      </c>
+      <c r="D133" t="n">
+        <v>11.791021</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="1" t="inlineStr">
+        <is>
+          <t>2023-01</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>7.397422</v>
+      </c>
+      <c r="C134" t="n">
+        <v>13593.482594</v>
+      </c>
+      <c r="D134" t="n">
+        <v>17.334022</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="1" t="inlineStr">
+        <is>
+          <t>2023-02</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>6.169563</v>
+      </c>
+      <c r="C135" t="n">
+        <v>11906.275882</v>
+      </c>
+      <c r="D135" t="n">
+        <v>14.959147</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="1" t="inlineStr">
+        <is>
+          <t>2023-03</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>4.255066</v>
+      </c>
+      <c r="C136" t="n">
+        <v>13996.904605</v>
+      </c>
+      <c r="D136" t="n">
+        <v>12.218202</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="1" t="inlineStr">
+        <is>
+          <t>2023-04</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>3.097191</v>
+      </c>
+      <c r="C137" t="n">
+        <v>10046.212478</v>
+      </c>
+      <c r="D137" t="n">
+        <v>10.445752</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="1" t="inlineStr">
+        <is>
+          <t>2023-05</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>3.203941</v>
+      </c>
+      <c r="C138" t="n">
+        <v>10815.469724</v>
+      </c>
+      <c r="D138" t="n">
+        <v>11.948274</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="1" t="inlineStr">
+        <is>
+          <t>2023-06</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>3.483265</v>
+      </c>
+      <c r="C139" t="n">
+        <v>12071.781236</v>
+      </c>
+      <c r="D139" t="n">
+        <v>13.475184</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="1" t="inlineStr">
+        <is>
+          <t>2023-07</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>4.075933</v>
+      </c>
+      <c r="C140" t="n">
+        <v>12477.225903</v>
+      </c>
+      <c r="D140" t="n">
+        <v>15.123414</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="1" t="inlineStr">
+        <is>
+          <t>2023-08</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>3.677969</v>
+      </c>
+      <c r="C141" t="n">
+        <v>11756.000499</v>
+      </c>
+      <c r="D141" t="n">
+        <v>13.465058</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="1" t="inlineStr">
+        <is>
+          <t>2023-09</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>3.307597</v>
+      </c>
+      <c r="C142" t="n">
+        <v>10962.244457</v>
+      </c>
+      <c r="D142" t="n">
+        <v>12.218237</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="1" t="inlineStr">
+        <is>
+          <t>2023-10</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>3.241957</v>
+      </c>
+      <c r="C143" t="n">
+        <v>10454.125794</v>
+      </c>
+      <c r="D143" t="n">
+        <v>11.581384</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="1" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>2.958686</v>
+      </c>
+      <c r="C144" t="n">
+        <v>11040.811143</v>
+      </c>
+      <c r="D144" t="n">
+        <v>9.912915999999999</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="1" t="inlineStr">
+        <is>
+          <t>2023-12</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>3.870235</v>
+      </c>
+      <c r="C145" t="n">
+        <v>11763.004028</v>
+      </c>
+      <c r="D145" t="n">
+        <v>11.588752</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="1" t="inlineStr">
+        <is>
+          <t>2024-01</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>7.039725000000001</v>
+      </c>
+      <c r="C146" t="n">
+        <v>13090.206981</v>
+      </c>
+      <c r="D146" t="n">
+        <v>17.147723</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="1" t="inlineStr">
+        <is>
+          <t>2024-02</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>6.126708000000001</v>
+      </c>
+      <c r="C147" t="n">
+        <v>12851.124118</v>
+      </c>
+      <c r="D147" t="n">
+        <v>15.254529</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="1" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>4.003228</v>
+      </c>
+      <c r="C148" t="n">
+        <v>11956.626841</v>
+      </c>
+      <c r="D148" t="n">
+        <v>11.582494</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="1" t="inlineStr">
+        <is>
+          <t>2024-04</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>2.878526</v>
+      </c>
+      <c r="C149" t="n">
+        <v>10004.921217</v>
+      </c>
+      <c r="D149" t="n">
+        <v>10.110105</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="1" t="inlineStr">
+        <is>
+          <t>2024-05</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>3.283046</v>
+      </c>
+      <c r="C150" t="n">
+        <v>12213.338451</v>
+      </c>
+      <c r="D150" t="n">
+        <v>12.41048</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="1" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>3.368335</v>
+      </c>
+      <c r="C151" t="n">
+        <v>11226.223824</v>
+      </c>
+      <c r="D151" t="n">
+        <v>12.772503</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="1" t="inlineStr">
+        <is>
+          <t>2024-07</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>4.053407</v>
+      </c>
+      <c r="C152" t="n">
+        <v>13226.304292</v>
+      </c>
+      <c r="D152" t="n">
+        <v>14.996078</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="1" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>3.478011</v>
+      </c>
+      <c r="C153" t="n">
+        <v>12171.606645</v>
+      </c>
+      <c r="D153" t="n">
+        <v>12.99697</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="1" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>2.87571</v>
+      </c>
+      <c r="C154" t="n">
+        <v>10237.192793</v>
+      </c>
+      <c r="D154" t="n">
+        <v>10.538912</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="1" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>2.954901</v>
+      </c>
+      <c r="C155" t="n">
+        <v>10678.921134</v>
+      </c>
+      <c r="D155" t="n">
+        <v>10.278138</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="1" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>2.952563</v>
+      </c>
+      <c r="C156" t="n">
+        <v>11064.005964</v>
+      </c>
+      <c r="D156" t="n">
+        <v>9.348742</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="1" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>3.782408</v>
+      </c>
+      <c r="C157" t="n">
+        <v>11498.928525</v>
+      </c>
+      <c r="D157" t="n">
+        <v>11.386739</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="1" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>7.005344</v>
+      </c>
+      <c r="C158" t="n">
+        <v>13605.512563</v>
+      </c>
+      <c r="D158" t="n">
+        <v>16.83577</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="1" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>5.941099</v>
+      </c>
+      <c r="C159" t="n">
+        <v>12908.058921</v>
+      </c>
+      <c r="D159" t="n">
+        <v>14.773244</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="1" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>4.092354</v>
+      </c>
+      <c r="C160" t="n">
+        <v>11653.169774</v>
+      </c>
+      <c r="D160" t="n">
+        <v>11.489983</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="1" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>3.124232</v>
+      </c>
+      <c r="C161" t="n">
+        <v>9822.824909999999</v>
+      </c>
+      <c r="D161" t="n">
+        <v>10.593454</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="1" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>3.05714</v>
+      </c>
+      <c r="C162" t="n">
+        <v>10944.561146</v>
+      </c>
+      <c r="D162" t="n">
+        <v>11.332466</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="1" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>3.602948</v>
+      </c>
+      <c r="C163" t="n">
+        <v>12685.14374</v>
+      </c>
+      <c r="D163" t="n">
+        <v>13.409062</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="1" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>4.062733000000001</v>
+      </c>
+      <c r="C164" t="n">
+        <v>12901.61855</v>
+      </c>
+      <c r="D164" t="n">
+        <v>14.722514</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="1" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>3.571546999999999</v>
+      </c>
+      <c r="C165" t="n">
+        <v>11718.756339</v>
+      </c>
+      <c r="D165" t="n">
+        <v>13.214027</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="1" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>3.173492</v>
+      </c>
+      <c r="C166" t="n">
+        <v>10631.54053</v>
+      </c>
+      <c r="D166" t="n">
+        <v>11.555475</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="1" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>2.989936</v>
+      </c>
+      <c r="C167" t="n">
+        <v>10591.335541</v>
+      </c>
+      <c r="D167" t="n">
+        <v>10.158655</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="1" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>3.126208</v>
+      </c>
+      <c r="C168" t="n">
+        <v>10711.334192</v>
+      </c>
+      <c r="D168" t="n">
+        <v>10.171583</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="1" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>4.14283</v>
+      </c>
+      <c r="C169" t="n">
+        <v>13077.047231</v>
+      </c>
+      <c r="D169" t="n">
+        <v>12.322182</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="1" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>6.802868999999999</v>
+      </c>
+      <c r="C170" t="n">
+        <v>13145.374526</v>
+      </c>
+      <c r="D170" t="n">
+        <v>16.557891</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="1" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>5.874545</v>
+      </c>
+      <c r="C171" t="n">
+        <v>11780.616317</v>
+      </c>
+      <c r="D171" t="n">
+        <v>14.251107</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="1" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>3.949008</v>
+      </c>
+      <c r="C172" t="n">
+        <v>11945.035338</v>
+      </c>
+      <c r="D172" t="n">
+        <v>11.299847</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="1" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>3.114791</v>
+      </c>
+      <c r="C173" t="n">
+        <v>10579.342832</v>
+      </c>
+      <c r="D173" t="n">
+        <v>10.161091</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="1" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>3.544113</v>
+      </c>
+      <c r="C174" t="n">
+        <v>12151.531183</v>
+      </c>
+      <c r="D174" t="n">
+        <v>12.794065</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="1" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>3.499194</v>
+      </c>
+      <c r="C175" t="n">
+        <v>12641.171137</v>
+      </c>
+      <c r="D175" t="n">
+        <v>13.163251</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="1" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>4.06659</v>
+      </c>
+      <c r="C176" t="n">
+        <v>13063.214629</v>
+      </c>
+      <c r="D176" t="n">
+        <v>14.820217</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="1" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>3.710309</v>
+      </c>
+      <c r="C177" t="n">
+        <v>12432.027715</v>
+      </c>
+      <c r="D177" t="n">
+        <v>13.547319</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr"/>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>verano</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>invierno</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>localidad</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>San Bernardo (La Costa)</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Total país</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Villa Gesell</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>San Bernardo (La Costa)</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Total país</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>Villa Gesell</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>fecha</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B4" t="n">
+        <v>71.31102736414799</v>
+      </c>
+      <c r="C4" t="n">
+        <v>86.76522420302851</v>
+      </c>
+      <c r="D4" t="n">
+        <v>93.78536012812008</v>
+      </c>
+      <c r="E4" t="n">
+        <v>91.39689542051376</v>
+      </c>
+      <c r="F4" t="n">
+        <v>91.80531374671163</v>
+      </c>
+      <c r="G4" t="n">
+        <v>92.47354756496502</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B5" t="n">
+        <v>69.34403264029262</v>
+      </c>
+      <c r="C5" t="n">
+        <v>87.08930140098329</v>
+      </c>
+      <c r="D5" t="n">
+        <v>93.07834651933155</v>
+      </c>
+      <c r="E5" t="n">
+        <v>96.59291030626912</v>
+      </c>
+      <c r="F5" t="n">
+        <v>93.70818433417386</v>
+      </c>
+      <c r="G5" t="n">
+        <v>96.44639864774018</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B6" t="n">
+        <v>82.89953353128969</v>
+      </c>
+      <c r="C6" t="n">
+        <v>90.66134069968825</v>
+      </c>
+      <c r="D6" t="n">
+        <v>95.23385311984644</v>
+      </c>
+      <c r="E6" t="n">
+        <v>91.45228709754227</v>
+      </c>
+      <c r="F6" t="n">
+        <v>94.67687993505109</v>
+      </c>
+      <c r="G6" t="n">
+        <v>91.78292737914289</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B7" t="n">
+        <v>95.47917893642169</v>
+      </c>
+      <c r="C7" t="n">
+        <v>92.9164872216619</v>
+      </c>
+      <c r="D7" t="n">
+        <v>98.97984420695214</v>
+      </c>
+      <c r="E7" t="n">
+        <v>93.5883665352699</v>
+      </c>
+      <c r="F7" t="n">
+        <v>99.11558564378034</v>
+      </c>
+      <c r="G7" t="n">
+        <v>96.94103647614948</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B8" t="n">
+        <v>100</v>
+      </c>
+      <c r="C8" t="n">
+        <v>100</v>
+      </c>
+      <c r="D8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E8" t="n">
+        <v>100</v>
+      </c>
+      <c r="F8" t="n">
+        <v>99.99999999999999</v>
+      </c>
+      <c r="G8" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B9" t="n">
+        <v>94.16644699070977</v>
+      </c>
+      <c r="C9" t="n">
+        <v>98.0188996353865</v>
+      </c>
+      <c r="D9" t="n">
+        <v>94.65487384408817</v>
+      </c>
+      <c r="E9" t="n">
+        <v>99.42294549238515</v>
+      </c>
+      <c r="F9" t="n">
+        <v>99.03165813020081</v>
+      </c>
+      <c r="G9" t="n">
+        <v>97.83588672268026</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B10" t="n">
+        <v>90.44175093457861</v>
+      </c>
+      <c r="C10" t="n">
+        <v>98.66107107849147</v>
+      </c>
+      <c r="D10" t="n">
+        <v>98.39481523988695</v>
+      </c>
+      <c r="E10" t="n">
+        <v>101.1780294011305</v>
+      </c>
+      <c r="F10" t="n">
+        <v>104.785471668589</v>
+      </c>
+      <c r="G10" t="n">
+        <v>102.3058550570662</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B11" t="n">
+        <v>75.59070896141989</v>
+      </c>
+      <c r="C11" t="n">
+        <v>93.0597748130776</v>
+      </c>
+      <c r="D11" t="n">
+        <v>94.01053567237794</v>
+      </c>
+      <c r="E11" t="n">
+        <v>96.48250174166864</v>
+      </c>
+      <c r="F11" t="n">
+        <v>98.61701290661155</v>
+      </c>
+      <c r="G11" t="n">
+        <v>83.26027223896345</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B12" t="n">
+        <v>69.82754716622313</v>
+      </c>
+      <c r="C12" t="n">
+        <v>94.85223286901785</v>
+      </c>
+      <c r="D12" t="n">
+        <v>97.0971135827161</v>
+      </c>
+      <c r="E12" t="n">
+        <v>93.46989999735446</v>
+      </c>
+      <c r="F12" t="n">
+        <v>97.38688130328866</v>
+      </c>
+      <c r="G12" t="n">
+        <v>91.8611044731237</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B13" t="n">
+        <v>51.10714802015779</v>
+      </c>
+      <c r="C13" t="n">
+        <v>91.50721755992673</v>
+      </c>
+      <c r="D13" t="n">
+        <v>81.02634203906671</v>
+      </c>
+      <c r="E13" t="n">
+        <v>109.0024427453989</v>
+      </c>
+      <c r="F13" t="n">
+        <v>104.436720252005</v>
+      </c>
+      <c r="G13" t="n">
+        <v>107.4778324513157</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B14" t="n">
+        <v>67.57956777763876</v>
+      </c>
+      <c r="C14" t="n">
+        <v>98.15524629613816</v>
+      </c>
+      <c r="D14" t="n">
+        <v>98.72911070172925</v>
+      </c>
+      <c r="E14" t="n">
+        <v>120.2306277943861</v>
+      </c>
+      <c r="F14" t="n">
+        <v>108.3682135246524</v>
+      </c>
+      <c r="G14" t="n">
+        <v>120.0318905513868</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B15" t="n">
+        <v>72.88380872607159</v>
+      </c>
+      <c r="C15" t="n">
+        <v>105.9102711428166</v>
+      </c>
+      <c r="D15" t="n">
+        <v>102.5531253403944</v>
+      </c>
+      <c r="E15" t="n">
+        <v>123.8697562545746</v>
+      </c>
+      <c r="F15" t="n">
+        <v>104.9337290159315</v>
+      </c>
+      <c r="G15" t="n">
+        <v>119.465755587038</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B16" t="n">
+        <v>70.73198535832664</v>
+      </c>
+      <c r="C16" t="n">
+        <v>107.7442915032522</v>
+      </c>
+      <c r="D16" t="n">
+        <v>102.8995392389965</v>
+      </c>
+      <c r="E16" t="n">
+        <v>120.1503677345962</v>
+      </c>
+      <c r="F16" t="n">
+        <v>105.856114141984</v>
+      </c>
+      <c r="G16" t="n">
+        <v>115.778983931804</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B17" t="n">
+        <v>69.55016721069482</v>
+      </c>
+      <c r="C17" t="n">
+        <v>110.1210251649165</v>
+      </c>
+      <c r="D17" t="n">
+        <v>100.3804604815427</v>
+      </c>
+      <c r="E17" t="n">
+        <v>123.8704286709525</v>
+      </c>
+      <c r="F17" t="n">
+        <v>107.8255435626709</v>
+      </c>
+      <c r="G17" t="n">
+        <v>117.4264001825401</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B18" t="n">
+        <v>68.10490445130013</v>
+      </c>
+      <c r="C18" t="n">
+        <v>103.527194234806</v>
+      </c>
+      <c r="D18" t="n">
+        <v>97.83985689066191</v>
+      </c>
+      <c r="E18" t="n">
+        <v>124.2988460894027</v>
+      </c>
+      <c r="F18" t="n">
+        <v>110.227110203556</v>
+      </c>
+      <c r="G18" t="n">
+        <v>117.9523446340312</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="E1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>